<commit_message>
Update: 0604-0607 real-time trading review data in statistics table
</commit_message>
<xml_diff>
--- a/02 Dayahead_Trading_Review/assets/输出模版-0505-日前机组组合收益复盘.xlsx
+++ b/02 Dayahead_Trading_Review/assets/输出模版-0505-日前机组组合收益复盘.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BaiduSyncdisk\01 电力交易与储能\01 各省项目及政策\04山东\每日策略实例\2026\05月\0505-晴天\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DataWork\Storage_Strategy\02 Dayahead_Trading_Review\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389D60C1-A860-42E5-8100-510F54A75BFF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CC2B104-B8B6-4AFF-B612-7156FA84807D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12252" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12252" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="充放测算" sheetId="1" r:id="rId1"/>
@@ -635,7 +635,7 @@
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
   <si>
-    <t>5月</t>
+    <t>6月</t>
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
 </sst>
@@ -1491,13 +1491,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1506,7 +1500,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4072,40 +4072,40 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0.3</c:v>
@@ -4120,76 +4120,76 @@
                   <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>0.1</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.3</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.3</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.3</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.3</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>1</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>1</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>1</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>1</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="64">
                   <c:v>2</c:v>
@@ -4240,40 +4240,40 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="80">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="88">
                   <c:v>1.7</c:v>
                 </c:pt>
-                <c:pt idx="81">
+                <c:pt idx="89">
                   <c:v>1.7</c:v>
                 </c:pt>
-                <c:pt idx="82">
+                <c:pt idx="90">
                   <c:v>1.7</c:v>
                 </c:pt>
-                <c:pt idx="83">
+                <c:pt idx="91">
                   <c:v>1.7</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>1.7</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>1.7</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>1.7</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>1.7</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="92">
                   <c:v>1</c:v>
@@ -6636,15 +6636,15 @@
       </c>
       <c r="I4" s="48">
         <f ca="1">B4*J4*70.5</f>
-        <v>-4436.2124999999996</v>
+        <v>-14223.375</v>
       </c>
       <c r="J4" s="48">
         <f ca="1">容量分摊系数!G3</f>
-        <v>0.35351123595505618</v>
+        <v>1.1334269662921348</v>
       </c>
       <c r="K4" s="54">
         <f ca="1">C4+D4+E4+F4+G4+H4+I4</f>
-        <v>7596.4443399999982</v>
+        <v>-2190.7181600000022</v>
       </c>
       <c r="L4" s="48">
         <f>报价及预中标!D26</f>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="O4" s="54">
         <f ca="1">N4+K4</f>
-        <v>71804.709140000006</v>
+        <v>62017.54664</v>
       </c>
       <c r="P4" s="58">
         <f>-M4/B4</f>
@@ -8000,7 +8000,7 @@
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D30" s="64">
         <f ca="1">充放测算!O4</f>
-        <v>71804.709140000006</v>
+        <v>62017.54664</v>
       </c>
       <c r="G30" s="43">
         <v>29</v>
@@ -10112,7 +10112,7 @@
       <c r="B3" s="7"/>
       <c r="C3" s="8">
         <f t="array" aca="1" ref="C3" ca="1">SUMPRODUCT(C8:C103,D8:D103)/SUM(C8:C103)</f>
-        <v>0.33750000000000002</v>
+        <v>1.125</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>162</v>
@@ -10120,7 +10120,7 @@
       <c r="F3" s="7"/>
       <c r="G3" s="8">
         <f t="array" aca="1" ref="G3" ca="1">SUMPRODUCT(D8:D103,E8:E103)/SUM(E8:E103)</f>
-        <v>0.35351123595505618</v>
+        <v>1.1334269662921348</v>
       </c>
       <c r="H3" s="84"/>
       <c r="J3" s="84"/>
@@ -10146,44 +10146,44 @@
       <c r="L5" s="84"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="93" t="s">
+      <c r="A6" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="93" t="s">
+      <c r="B6" s="91" t="s">
         <v>163</v>
       </c>
-      <c r="C6" s="93" t="s">
+      <c r="C6" s="91" t="s">
         <v>164</v>
       </c>
       <c r="D6" s="82" t="s">
         <v>165</v>
       </c>
-      <c r="E6" s="93" t="s">
+      <c r="E6" s="91" t="s">
         <v>166</v>
       </c>
-      <c r="F6" s="90" t="s">
+      <c r="F6" s="93" t="s">
         <v>181</v>
       </c>
-      <c r="G6" s="91"/>
-      <c r="H6" s="91"/>
-      <c r="I6" s="91"/>
-      <c r="J6" s="91"/>
-      <c r="K6" s="91"/>
-      <c r="L6" s="91"/>
-      <c r="M6" s="91"/>
-      <c r="N6" s="91"/>
-      <c r="O6" s="91"/>
-      <c r="P6" s="91"/>
-      <c r="Q6" s="92"/>
+      <c r="G6" s="94"/>
+      <c r="H6" s="94"/>
+      <c r="I6" s="94"/>
+      <c r="J6" s="94"/>
+      <c r="K6" s="94"/>
+      <c r="L6" s="94"/>
+      <c r="M6" s="94"/>
+      <c r="N6" s="94"/>
+      <c r="O6" s="94"/>
+      <c r="P6" s="94"/>
+      <c r="Q6" s="95"/>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="94"/>
-      <c r="B7" s="94"/>
-      <c r="C7" s="94"/>
+      <c r="A7" s="92"/>
+      <c r="B7" s="92"/>
+      <c r="C7" s="92"/>
       <c r="D7" s="63" t="s">
         <v>182</v>
       </c>
-      <c r="E7" s="94"/>
+      <c r="E7" s="92"/>
       <c r="F7" s="12" t="s">
         <v>168</v>
       </c>
@@ -10222,7 +10222,7 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="95">
+      <c r="A8" s="90">
         <v>1</v>
       </c>
       <c r="B8" s="83">
@@ -10278,7 +10278,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="95"/>
+      <c r="A9" s="90"/>
       <c r="B9" s="83">
         <v>2</v>
       </c>
@@ -10332,7 +10332,7 @@
       </c>
     </row>
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="95"/>
+      <c r="A10" s="90"/>
       <c r="B10" s="83">
         <v>3</v>
       </c>
@@ -10386,7 +10386,7 @@
       </c>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="95"/>
+      <c r="A11" s="90"/>
       <c r="B11" s="83">
         <v>4</v>
       </c>
@@ -10440,7 +10440,7 @@
       </c>
     </row>
     <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="95">
+      <c r="A12" s="90">
         <v>2</v>
       </c>
       <c r="B12" s="83">
@@ -10496,7 +10496,7 @@
       </c>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="95"/>
+      <c r="A13" s="90"/>
       <c r="B13" s="83">
         <v>6</v>
       </c>
@@ -10550,7 +10550,7 @@
       </c>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="95"/>
+      <c r="A14" s="90"/>
       <c r="B14" s="83">
         <v>7</v>
       </c>
@@ -10604,7 +10604,7 @@
       </c>
     </row>
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="95"/>
+      <c r="A15" s="90"/>
       <c r="B15" s="83">
         <v>8</v>
       </c>
@@ -10658,7 +10658,7 @@
       </c>
     </row>
     <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="95">
+      <c r="A16" s="90">
         <v>3</v>
       </c>
       <c r="B16" s="83">
@@ -10714,7 +10714,7 @@
       </c>
     </row>
     <row r="17" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="95"/>
+      <c r="A17" s="90"/>
       <c r="B17" s="83">
         <v>10</v>
       </c>
@@ -10768,7 +10768,7 @@
       </c>
     </row>
     <row r="18" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="95"/>
+      <c r="A18" s="90"/>
       <c r="B18" s="83">
         <v>11</v>
       </c>
@@ -10822,7 +10822,7 @@
       </c>
     </row>
     <row r="19" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="95"/>
+      <c r="A19" s="90"/>
       <c r="B19" s="83">
         <v>12</v>
       </c>
@@ -10876,7 +10876,7 @@
       </c>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="95">
+      <c r="A20" s="90">
         <v>4</v>
       </c>
       <c r="B20" s="83">
@@ -10932,7 +10932,7 @@
       </c>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="95"/>
+      <c r="A21" s="90"/>
       <c r="B21" s="83">
         <v>14</v>
       </c>
@@ -10986,7 +10986,7 @@
       </c>
     </row>
     <row r="22" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="95"/>
+      <c r="A22" s="90"/>
       <c r="B22" s="83">
         <v>15</v>
       </c>
@@ -11040,7 +11040,7 @@
       </c>
     </row>
     <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="95"/>
+      <c r="A23" s="90"/>
       <c r="B23" s="83">
         <v>16</v>
       </c>
@@ -11094,7 +11094,7 @@
       </c>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="95">
+      <c r="A24" s="90">
         <v>5</v>
       </c>
       <c r="B24" s="83">
@@ -11150,7 +11150,7 @@
       </c>
     </row>
     <row r="25" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="95"/>
+      <c r="A25" s="90"/>
       <c r="B25" s="83">
         <v>18</v>
       </c>
@@ -11204,7 +11204,7 @@
       </c>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="95"/>
+      <c r="A26" s="90"/>
       <c r="B26" s="83">
         <v>19</v>
       </c>
@@ -11258,7 +11258,7 @@
       </c>
     </row>
     <row r="27" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="95"/>
+      <c r="A27" s="90"/>
       <c r="B27" s="83">
         <v>20</v>
       </c>
@@ -11312,7 +11312,7 @@
       </c>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="95">
+      <c r="A28" s="90">
         <v>6</v>
       </c>
       <c r="B28" s="83">
@@ -11368,7 +11368,7 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="95"/>
+      <c r="A29" s="90"/>
       <c r="B29" s="83">
         <v>22</v>
       </c>
@@ -11422,7 +11422,7 @@
       </c>
     </row>
     <row r="30" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="95"/>
+      <c r="A30" s="90"/>
       <c r="B30" s="83">
         <v>23</v>
       </c>
@@ -11476,7 +11476,7 @@
       </c>
     </row>
     <row r="31" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="95"/>
+      <c r="A31" s="90"/>
       <c r="B31" s="83">
         <v>24</v>
       </c>
@@ -11530,7 +11530,7 @@
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="95">
+      <c r="A32" s="90">
         <v>7</v>
       </c>
       <c r="B32" s="83">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="D32" s="83">
         <f t="array" aca="1" ref="D32" ca="1">INDIRECT(ADDRESS(B32+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E32" s="13">
         <f>报价及预中标!L26/4</f>
@@ -11586,7 +11586,7 @@
       </c>
     </row>
     <row r="33" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="95"/>
+      <c r="A33" s="90"/>
       <c r="B33" s="83">
         <v>26</v>
       </c>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="D33" s="83">
         <f t="array" aca="1" ref="D33" ca="1">INDIRECT(ADDRESS(B33+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E33" s="13">
         <f>报价及预中标!L27/4</f>
@@ -11640,7 +11640,7 @@
       </c>
     </row>
     <row r="34" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="95"/>
+      <c r="A34" s="90"/>
       <c r="B34" s="83">
         <v>27</v>
       </c>
@@ -11650,7 +11650,7 @@
       </c>
       <c r="D34" s="83">
         <f t="array" aca="1" ref="D34" ca="1">INDIRECT(ADDRESS(B34+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E34" s="13">
         <f>报价及预中标!L28/4</f>
@@ -11694,7 +11694,7 @@
       </c>
     </row>
     <row r="35" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="95"/>
+      <c r="A35" s="90"/>
       <c r="B35" s="83">
         <v>28</v>
       </c>
@@ -11704,7 +11704,7 @@
       </c>
       <c r="D35" s="83">
         <f t="array" aca="1" ref="D35" ca="1">INDIRECT(ADDRESS(B35+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E35" s="13">
         <f>报价及预中标!L29/4</f>
@@ -11748,7 +11748,7 @@
       </c>
     </row>
     <row r="36" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="95">
+      <c r="A36" s="90">
         <v>8</v>
       </c>
       <c r="B36" s="83">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="D36" s="83">
         <f t="array" aca="1" ref="D36" ca="1">INDIRECT(ADDRESS(B36+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E36" s="13">
         <f>报价及预中标!L30/4</f>
@@ -11804,7 +11804,7 @@
       </c>
     </row>
     <row r="37" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="95"/>
+      <c r="A37" s="90"/>
       <c r="B37" s="83">
         <v>30</v>
       </c>
@@ -11814,7 +11814,7 @@
       </c>
       <c r="D37" s="83">
         <f t="array" aca="1" ref="D37" ca="1">INDIRECT(ADDRESS(B37+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E37" s="13">
         <f>报价及预中标!L31/4</f>
@@ -11858,7 +11858,7 @@
       </c>
     </row>
     <row r="38" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="95"/>
+      <c r="A38" s="90"/>
       <c r="B38" s="83">
         <v>31</v>
       </c>
@@ -11868,7 +11868,7 @@
       </c>
       <c r="D38" s="83">
         <f t="array" aca="1" ref="D38" ca="1">INDIRECT(ADDRESS(B38+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E38" s="13">
         <f>报价及预中标!L32/4</f>
@@ -11912,7 +11912,7 @@
       </c>
     </row>
     <row r="39" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="95"/>
+      <c r="A39" s="90"/>
       <c r="B39" s="83">
         <v>32</v>
       </c>
@@ -11922,7 +11922,7 @@
       </c>
       <c r="D39" s="83">
         <f t="array" aca="1" ref="D39" ca="1">INDIRECT(ADDRESS(B39+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E39" s="13">
         <f>报价及预中标!L33/4</f>
@@ -11966,7 +11966,7 @@
       </c>
     </row>
     <row r="40" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="95">
+      <c r="A40" s="90">
         <v>9</v>
       </c>
       <c r="B40" s="83">
@@ -11978,7 +11978,7 @@
       </c>
       <c r="D40" s="83">
         <f t="array" aca="1" ref="D40" ca="1">INDIRECT(ADDRESS(B40+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E40" s="13">
         <f>报价及预中标!L34/4</f>
@@ -12022,7 +12022,7 @@
       </c>
     </row>
     <row r="41" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="95"/>
+      <c r="A41" s="90"/>
       <c r="B41" s="83">
         <v>34</v>
       </c>
@@ -12032,7 +12032,7 @@
       </c>
       <c r="D41" s="83">
         <f t="array" aca="1" ref="D41" ca="1">INDIRECT(ADDRESS(B41+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E41" s="13">
         <f>报价及预中标!L35/4</f>
@@ -12076,7 +12076,7 @@
       </c>
     </row>
     <row r="42" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="95"/>
+      <c r="A42" s="90"/>
       <c r="B42" s="83">
         <v>35</v>
       </c>
@@ -12086,7 +12086,7 @@
       </c>
       <c r="D42" s="83">
         <f t="array" aca="1" ref="D42" ca="1">INDIRECT(ADDRESS(B42+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E42" s="13">
         <f>报价及预中标!L36/4</f>
@@ -12130,7 +12130,7 @@
       </c>
     </row>
     <row r="43" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="95"/>
+      <c r="A43" s="90"/>
       <c r="B43" s="83">
         <v>36</v>
       </c>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="D43" s="83">
         <f t="array" aca="1" ref="D43" ca="1">INDIRECT(ADDRESS(B43+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E43" s="13">
         <f>报价及预中标!L37/4</f>
@@ -12184,7 +12184,7 @@
       </c>
     </row>
     <row r="44" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="95">
+      <c r="A44" s="90">
         <v>10</v>
       </c>
       <c r="B44" s="83">
@@ -12240,7 +12240,7 @@
       </c>
     </row>
     <row r="45" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="95"/>
+      <c r="A45" s="90"/>
       <c r="B45" s="83">
         <v>38</v>
       </c>
@@ -12294,7 +12294,7 @@
       </c>
     </row>
     <row r="46" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="95"/>
+      <c r="A46" s="90"/>
       <c r="B46" s="83">
         <v>39</v>
       </c>
@@ -12348,7 +12348,7 @@
       </c>
     </row>
     <row r="47" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="95"/>
+      <c r="A47" s="90"/>
       <c r="B47" s="83">
         <v>40</v>
       </c>
@@ -12402,7 +12402,7 @@
       </c>
     </row>
     <row r="48" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="95">
+      <c r="A48" s="90">
         <v>11</v>
       </c>
       <c r="B48" s="83">
@@ -12414,7 +12414,7 @@
       </c>
       <c r="D48" s="83">
         <f t="array" aca="1" ref="D48" ca="1">INDIRECT(ADDRESS(B48+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E48" s="13">
         <f>报价及预中标!L42/4</f>
@@ -12458,7 +12458,7 @@
       </c>
     </row>
     <row r="49" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="95"/>
+      <c r="A49" s="90"/>
       <c r="B49" s="83">
         <v>42</v>
       </c>
@@ -12468,7 +12468,7 @@
       </c>
       <c r="D49" s="83">
         <f t="array" aca="1" ref="D49" ca="1">INDIRECT(ADDRESS(B49+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E49" s="13">
         <f>报价及预中标!L43/4</f>
@@ -12512,7 +12512,7 @@
       </c>
     </row>
     <row r="50" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="95"/>
+      <c r="A50" s="90"/>
       <c r="B50" s="83">
         <v>43</v>
       </c>
@@ -12522,7 +12522,7 @@
       </c>
       <c r="D50" s="83">
         <f t="array" aca="1" ref="D50" ca="1">INDIRECT(ADDRESS(B50+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E50" s="13">
         <f>报价及预中标!L44/4</f>
@@ -12566,7 +12566,7 @@
       </c>
     </row>
     <row r="51" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="95"/>
+      <c r="A51" s="90"/>
       <c r="B51" s="83">
         <v>44</v>
       </c>
@@ -12576,7 +12576,7 @@
       </c>
       <c r="D51" s="83">
         <f t="array" aca="1" ref="D51" ca="1">INDIRECT(ADDRESS(B51+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E51" s="13">
         <f>报价及预中标!L45/4</f>
@@ -12620,7 +12620,7 @@
       </c>
     </row>
     <row r="52" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="95">
+      <c r="A52" s="90">
         <v>12</v>
       </c>
       <c r="B52" s="83">
@@ -12632,7 +12632,7 @@
       </c>
       <c r="D52" s="83">
         <f t="array" aca="1" ref="D52" ca="1">INDIRECT(ADDRESS(B52+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E52" s="13">
         <f>报价及预中标!L46/4</f>
@@ -12676,7 +12676,7 @@
       </c>
     </row>
     <row r="53" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="95"/>
+      <c r="A53" s="90"/>
       <c r="B53" s="83">
         <v>46</v>
       </c>
@@ -12686,7 +12686,7 @@
       </c>
       <c r="D53" s="83">
         <f t="array" aca="1" ref="D53" ca="1">INDIRECT(ADDRESS(B53+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E53" s="13">
         <f>报价及预中标!L47/4</f>
@@ -12730,7 +12730,7 @@
       </c>
     </row>
     <row r="54" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="95"/>
+      <c r="A54" s="90"/>
       <c r="B54" s="83">
         <v>47</v>
       </c>
@@ -12740,7 +12740,7 @@
       </c>
       <c r="D54" s="83">
         <f t="array" aca="1" ref="D54" ca="1">INDIRECT(ADDRESS(B54+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E54" s="13">
         <f>报价及预中标!L48/4</f>
@@ -12784,7 +12784,7 @@
       </c>
     </row>
     <row r="55" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="95"/>
+      <c r="A55" s="90"/>
       <c r="B55" s="83">
         <v>48</v>
       </c>
@@ -12794,7 +12794,7 @@
       </c>
       <c r="D55" s="83">
         <f t="array" aca="1" ref="D55" ca="1">INDIRECT(ADDRESS(B55+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E55" s="13">
         <f>报价及预中标!L49/4</f>
@@ -12838,7 +12838,7 @@
       </c>
     </row>
     <row r="56" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="95">
+      <c r="A56" s="90">
         <v>13</v>
       </c>
       <c r="B56" s="83">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="D56" s="83">
         <f t="array" aca="1" ref="D56" ca="1">INDIRECT(ADDRESS(B56+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E56" s="13">
         <f>报价及预中标!L50/4</f>
@@ -12894,7 +12894,7 @@
       </c>
     </row>
     <row r="57" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="95"/>
+      <c r="A57" s="90"/>
       <c r="B57" s="83">
         <v>50</v>
       </c>
@@ -12904,7 +12904,7 @@
       </c>
       <c r="D57" s="83">
         <f t="array" aca="1" ref="D57" ca="1">INDIRECT(ADDRESS(B57+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E57" s="13">
         <f>报价及预中标!L51/4</f>
@@ -12948,7 +12948,7 @@
       </c>
     </row>
     <row r="58" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="95"/>
+      <c r="A58" s="90"/>
       <c r="B58" s="83">
         <v>51</v>
       </c>
@@ -12958,7 +12958,7 @@
       </c>
       <c r="D58" s="83">
         <f t="array" aca="1" ref="D58" ca="1">INDIRECT(ADDRESS(B58+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E58" s="13">
         <f>报价及预中标!L52/4</f>
@@ -13002,7 +13002,7 @@
       </c>
     </row>
     <row r="59" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="95"/>
+      <c r="A59" s="90"/>
       <c r="B59" s="83">
         <v>52</v>
       </c>
@@ -13012,7 +13012,7 @@
       </c>
       <c r="D59" s="83">
         <f t="array" aca="1" ref="D59" ca="1">INDIRECT(ADDRESS(B59+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E59" s="13">
         <f>报价及预中标!L53/4</f>
@@ -13056,7 +13056,7 @@
       </c>
     </row>
     <row r="60" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="95">
+      <c r="A60" s="90">
         <v>14</v>
       </c>
       <c r="B60" s="83">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="D60" s="83">
         <f t="array" aca="1" ref="D60" ca="1">INDIRECT(ADDRESS(B60+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E60" s="13">
         <f>报价及预中标!L54/4</f>
@@ -13112,7 +13112,7 @@
       </c>
     </row>
     <row r="61" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="95"/>
+      <c r="A61" s="90"/>
       <c r="B61" s="83">
         <v>54</v>
       </c>
@@ -13122,7 +13122,7 @@
       </c>
       <c r="D61" s="83">
         <f t="array" aca="1" ref="D61" ca="1">INDIRECT(ADDRESS(B61+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E61" s="13">
         <f>报价及预中标!L55/4</f>
@@ -13166,7 +13166,7 @@
       </c>
     </row>
     <row r="62" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="95"/>
+      <c r="A62" s="90"/>
       <c r="B62" s="83">
         <v>55</v>
       </c>
@@ -13176,7 +13176,7 @@
       </c>
       <c r="D62" s="83">
         <f t="array" aca="1" ref="D62" ca="1">INDIRECT(ADDRESS(B62+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E62" s="13">
         <f>报价及预中标!L56/4</f>
@@ -13220,7 +13220,7 @@
       </c>
     </row>
     <row r="63" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="95"/>
+      <c r="A63" s="90"/>
       <c r="B63" s="83">
         <v>56</v>
       </c>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="D63" s="83">
         <f t="array" aca="1" ref="D63" ca="1">INDIRECT(ADDRESS(B63+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E63" s="13">
         <f>报价及预中标!L57/4</f>
@@ -13274,7 +13274,7 @@
       </c>
     </row>
     <row r="64" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="95">
+      <c r="A64" s="90">
         <v>15</v>
       </c>
       <c r="B64" s="83">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="D64" s="83">
         <f t="array" aca="1" ref="D64" ca="1">INDIRECT(ADDRESS(B64+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E64" s="13">
         <f>报价及预中标!L58/4</f>
@@ -13330,7 +13330,7 @@
       </c>
     </row>
     <row r="65" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="95"/>
+      <c r="A65" s="90"/>
       <c r="B65" s="83">
         <v>58</v>
       </c>
@@ -13340,7 +13340,7 @@
       </c>
       <c r="D65" s="83">
         <f t="array" aca="1" ref="D65" ca="1">INDIRECT(ADDRESS(B65+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E65" s="13">
         <f>报价及预中标!L59/4</f>
@@ -13384,7 +13384,7 @@
       </c>
     </row>
     <row r="66" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="95"/>
+      <c r="A66" s="90"/>
       <c r="B66" s="83">
         <v>59</v>
       </c>
@@ -13394,7 +13394,7 @@
       </c>
       <c r="D66" s="83">
         <f t="array" aca="1" ref="D66" ca="1">INDIRECT(ADDRESS(B66+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E66" s="13">
         <f>报价及预中标!L60/4</f>
@@ -13438,7 +13438,7 @@
       </c>
     </row>
     <row r="67" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="95"/>
+      <c r="A67" s="90"/>
       <c r="B67" s="83">
         <v>60</v>
       </c>
@@ -13448,7 +13448,7 @@
       </c>
       <c r="D67" s="83">
         <f t="array" aca="1" ref="D67" ca="1">INDIRECT(ADDRESS(B67+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E67" s="13">
         <f>报价及预中标!L61/4</f>
@@ -13492,7 +13492,7 @@
       </c>
     </row>
     <row r="68" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="95">
+      <c r="A68" s="90">
         <v>16</v>
       </c>
       <c r="B68" s="83">
@@ -13504,7 +13504,7 @@
       </c>
       <c r="D68" s="83">
         <f t="array" aca="1" ref="D68" ca="1">INDIRECT(ADDRESS(B68+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="13">
         <f>报价及预中标!L62/4</f>
@@ -13548,7 +13548,7 @@
       </c>
     </row>
     <row r="69" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="95"/>
+      <c r="A69" s="90"/>
       <c r="B69" s="83">
         <v>62</v>
       </c>
@@ -13558,7 +13558,7 @@
       </c>
       <c r="D69" s="83">
         <f t="array" aca="1" ref="D69" ca="1">INDIRECT(ADDRESS(B69+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E69" s="13">
         <f>报价及预中标!L63/4</f>
@@ -13602,7 +13602,7 @@
       </c>
     </row>
     <row r="70" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="95"/>
+      <c r="A70" s="90"/>
       <c r="B70" s="83">
         <v>63</v>
       </c>
@@ -13612,7 +13612,7 @@
       </c>
       <c r="D70" s="83">
         <f t="array" aca="1" ref="D70" ca="1">INDIRECT(ADDRESS(B70+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E70" s="13">
         <f>报价及预中标!L64/4</f>
@@ -13656,7 +13656,7 @@
       </c>
     </row>
     <row r="71" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="95"/>
+      <c r="A71" s="90"/>
       <c r="B71" s="83">
         <v>64</v>
       </c>
@@ -13666,7 +13666,7 @@
       </c>
       <c r="D71" s="83">
         <f t="array" aca="1" ref="D71" ca="1">INDIRECT(ADDRESS(B71+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E71" s="13">
         <f>报价及预中标!L65/4</f>
@@ -13710,7 +13710,7 @@
       </c>
     </row>
     <row r="72" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="95">
+      <c r="A72" s="90">
         <v>17</v>
       </c>
       <c r="B72" s="83">
@@ -13766,7 +13766,7 @@
       </c>
     </row>
     <row r="73" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="95"/>
+      <c r="A73" s="90"/>
       <c r="B73" s="83">
         <v>66</v>
       </c>
@@ -13820,7 +13820,7 @@
       </c>
     </row>
     <row r="74" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="95"/>
+      <c r="A74" s="90"/>
       <c r="B74" s="83">
         <v>67</v>
       </c>
@@ -13874,7 +13874,7 @@
       </c>
     </row>
     <row r="75" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="95"/>
+      <c r="A75" s="90"/>
       <c r="B75" s="83">
         <v>68</v>
       </c>
@@ -13928,7 +13928,7 @@
       </c>
     </row>
     <row r="76" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="95">
+      <c r="A76" s="90">
         <v>18</v>
       </c>
       <c r="B76" s="83">
@@ -13984,7 +13984,7 @@
       </c>
     </row>
     <row r="77" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="95"/>
+      <c r="A77" s="90"/>
       <c r="B77" s="83">
         <v>70</v>
       </c>
@@ -14038,7 +14038,7 @@
       </c>
     </row>
     <row r="78" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="95"/>
+      <c r="A78" s="90"/>
       <c r="B78" s="83">
         <v>71</v>
       </c>
@@ -14092,7 +14092,7 @@
       </c>
     </row>
     <row r="79" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="95"/>
+      <c r="A79" s="90"/>
       <c r="B79" s="83">
         <v>72</v>
       </c>
@@ -14146,7 +14146,7 @@
       </c>
     </row>
     <row r="80" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="95">
+      <c r="A80" s="90">
         <v>19</v>
       </c>
       <c r="B80" s="83">
@@ -14202,7 +14202,7 @@
       </c>
     </row>
     <row r="81" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="95"/>
+      <c r="A81" s="90"/>
       <c r="B81" s="83">
         <v>74</v>
       </c>
@@ -14256,7 +14256,7 @@
       </c>
     </row>
     <row r="82" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="95"/>
+      <c r="A82" s="90"/>
       <c r="B82" s="83">
         <v>75</v>
       </c>
@@ -14310,7 +14310,7 @@
       </c>
     </row>
     <row r="83" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="95"/>
+      <c r="A83" s="90"/>
       <c r="B83" s="83">
         <v>76</v>
       </c>
@@ -14364,7 +14364,7 @@
       </c>
     </row>
     <row r="84" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="95">
+      <c r="A84" s="90">
         <v>20</v>
       </c>
       <c r="B84" s="83">
@@ -14420,7 +14420,7 @@
       </c>
     </row>
     <row r="85" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="95"/>
+      <c r="A85" s="90"/>
       <c r="B85" s="83">
         <v>78</v>
       </c>
@@ -14474,7 +14474,7 @@
       </c>
     </row>
     <row r="86" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="95"/>
+      <c r="A86" s="90"/>
       <c r="B86" s="83">
         <v>79</v>
       </c>
@@ -14528,7 +14528,7 @@
       </c>
     </row>
     <row r="87" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="95"/>
+      <c r="A87" s="90"/>
       <c r="B87" s="83">
         <v>80</v>
       </c>
@@ -14582,7 +14582,7 @@
       </c>
     </row>
     <row r="88" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="95">
+      <c r="A88" s="90">
         <v>21</v>
       </c>
       <c r="B88" s="83">
@@ -14594,7 +14594,7 @@
       </c>
       <c r="D88" s="83">
         <f t="array" aca="1" ref="D88" ca="1">INDIRECT(ADDRESS(B88+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E88" s="13">
         <f>报价及预中标!L82/4</f>
@@ -14638,7 +14638,7 @@
       </c>
     </row>
     <row r="89" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="95"/>
+      <c r="A89" s="90"/>
       <c r="B89" s="83">
         <v>82</v>
       </c>
@@ -14648,7 +14648,7 @@
       </c>
       <c r="D89" s="83">
         <f t="array" aca="1" ref="D89" ca="1">INDIRECT(ADDRESS(B89+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E89" s="13">
         <f>报价及预中标!L83/4</f>
@@ -14692,7 +14692,7 @@
       </c>
     </row>
     <row r="90" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="95"/>
+      <c r="A90" s="90"/>
       <c r="B90" s="83">
         <v>83</v>
       </c>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="D90" s="83">
         <f t="array" aca="1" ref="D90" ca="1">INDIRECT(ADDRESS(B90+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E90" s="13">
         <f>报价及预中标!L84/4</f>
@@ -14746,7 +14746,7 @@
       </c>
     </row>
     <row r="91" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="95"/>
+      <c r="A91" s="90"/>
       <c r="B91" s="83">
         <v>84</v>
       </c>
@@ -14756,7 +14756,7 @@
       </c>
       <c r="D91" s="83">
         <f t="array" aca="1" ref="D91" ca="1">INDIRECT(ADDRESS(B91+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E91" s="13">
         <f>报价及预中标!L85/4</f>
@@ -14800,7 +14800,7 @@
       </c>
     </row>
     <row r="92" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="95">
+      <c r="A92" s="90">
         <v>22</v>
       </c>
       <c r="B92" s="83">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="D92" s="83">
         <f t="array" aca="1" ref="D92" ca="1">INDIRECT(ADDRESS(B92+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E92" s="13">
         <f>报价及预中标!L86/4</f>
@@ -14856,7 +14856,7 @@
       </c>
     </row>
     <row r="93" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="95"/>
+      <c r="A93" s="90"/>
       <c r="B93" s="83">
         <v>86</v>
       </c>
@@ -14866,7 +14866,7 @@
       </c>
       <c r="D93" s="83">
         <f t="array" aca="1" ref="D93" ca="1">INDIRECT(ADDRESS(B93+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E93" s="13">
         <f>报价及预中标!L87/4</f>
@@ -14910,7 +14910,7 @@
       </c>
     </row>
     <row r="94" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="95"/>
+      <c r="A94" s="90"/>
       <c r="B94" s="83">
         <v>87</v>
       </c>
@@ -14920,7 +14920,7 @@
       </c>
       <c r="D94" s="83">
         <f t="array" aca="1" ref="D94" ca="1">INDIRECT(ADDRESS(B94+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E94" s="13">
         <f>报价及预中标!L88/4</f>
@@ -14964,7 +14964,7 @@
       </c>
     </row>
     <row r="95" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="95"/>
+      <c r="A95" s="90"/>
       <c r="B95" s="83">
         <v>88</v>
       </c>
@@ -14974,7 +14974,7 @@
       </c>
       <c r="D95" s="83">
         <f t="array" aca="1" ref="D95" ca="1">INDIRECT(ADDRESS(B95+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E95" s="13">
         <f>报价及预中标!L89/4</f>
@@ -15018,7 +15018,7 @@
       </c>
     </row>
     <row r="96" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="95">
+      <c r="A96" s="90">
         <v>23</v>
       </c>
       <c r="B96" s="83">
@@ -15030,7 +15030,7 @@
       </c>
       <c r="D96" s="83">
         <f t="array" aca="1" ref="D96" ca="1">INDIRECT(ADDRESS(B96+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E96" s="13">
         <f>报价及预中标!L90/4</f>
@@ -15074,7 +15074,7 @@
       </c>
     </row>
     <row r="97" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="95"/>
+      <c r="A97" s="90"/>
       <c r="B97" s="83">
         <v>90</v>
       </c>
@@ -15084,7 +15084,7 @@
       </c>
       <c r="D97" s="83">
         <f t="array" aca="1" ref="D97" ca="1">INDIRECT(ADDRESS(B97+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E97" s="13">
         <f>报价及预中标!L91/4</f>
@@ -15128,7 +15128,7 @@
       </c>
     </row>
     <row r="98" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="95"/>
+      <c r="A98" s="90"/>
       <c r="B98" s="83">
         <v>91</v>
       </c>
@@ -15138,7 +15138,7 @@
       </c>
       <c r="D98" s="83">
         <f t="array" aca="1" ref="D98" ca="1">INDIRECT(ADDRESS(B98+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E98" s="13">
         <f>报价及预中标!L92/4</f>
@@ -15182,7 +15182,7 @@
       </c>
     </row>
     <row r="99" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="95"/>
+      <c r="A99" s="90"/>
       <c r="B99" s="83">
         <v>92</v>
       </c>
@@ -15192,7 +15192,7 @@
       </c>
       <c r="D99" s="83">
         <f t="array" aca="1" ref="D99" ca="1">INDIRECT(ADDRESS(B99+ROW($D$7),MATCH($D$7,$F$7:$Q$7,0)+5))</f>
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E99" s="13">
         <f>报价及预中标!L93/4</f>
@@ -15236,7 +15236,7 @@
       </c>
     </row>
     <row r="100" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="95">
+      <c r="A100" s="90">
         <v>24</v>
       </c>
       <c r="B100" s="83">
@@ -15292,7 +15292,7 @@
       </c>
     </row>
     <row r="101" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="95"/>
+      <c r="A101" s="90"/>
       <c r="B101" s="83">
         <v>94</v>
       </c>
@@ -15346,7 +15346,7 @@
       </c>
     </row>
     <row r="102" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="95"/>
+      <c r="A102" s="90"/>
       <c r="B102" s="83">
         <v>95</v>
       </c>
@@ -15400,7 +15400,7 @@
       </c>
     </row>
     <row r="103" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="95"/>
+      <c r="A103" s="90"/>
       <c r="B103" s="83">
         <v>96</v>
       </c>
@@ -15455,6 +15455,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="F6:Q6"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A48:A51"/>
+    <mergeCell ref="A52:A55"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="A36:A39"/>
     <mergeCell ref="A100:A103"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
@@ -15471,19 +15484,6 @@
     <mergeCell ref="A76:A79"/>
     <mergeCell ref="A40:A43"/>
     <mergeCell ref="A44:A47"/>
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="A52:A55"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="A36:A39"/>
-    <mergeCell ref="F6:Q6"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A16:A19"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>